<commit_message>
updated UI of hotel-upload
</commit_message>
<xml_diff>
--- a/public/hotel_data_upload_v2.xlsx
+++ b/public/hotel_data_upload_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Rushi\internship manual\project\next_adwait_tour\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD7ECA8-8E32-418D-BFC0-397150CB18FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E379F67-7A13-46DB-92EC-799187D61483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1195,7 +1195,7 @@
         <v>0</v>
       </c>
       <c r="Z5" s="6">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3252,17 +3252,17 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="S1:V1"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="F1:F2"/>
     <mergeCell ref="W1:Z1"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="O1:R1"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="S1:V1"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="F1:F2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="D1:D2"/>

</xml_diff>